<commit_message>
Barranquita: caratula con SERVICIO DE DISEÑO - DRENAJE PLUVIAL en lugar de EXPEDIENTE TÉCNICO
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0142t8T16igb3VKxUPwnQPq6
</commit_message>
<xml_diff>
--- a/entregables_barranquita/ANALISIS_ESTADISTICO_IE0590_BARRANQUITA.xlsx
+++ b/entregables_barranquita/ANALISIS_ESTADISTICO_IE0590_BARRANQUITA.xlsx
@@ -68,7 +68,7 @@
     <t xml:space="preserve">GERENCIA TERRITORIAL BAJO MAYO - TARAPOTO</t>
   </si>
   <si>
-    <t xml:space="preserve">EXPEDIENTE TÉCNICO</t>
+    <t xml:space="preserve">SERVICIO DE DISEÑO - DRENAJE PLUVIAL</t>
   </si>
   <si>
     <t xml:space="preserve">“MEJORAMIENTO Y AMPLIACIÓN DEL SERVICIO DE EDUCACIÓN PRIMARIA EN I.E. N° 0590 DISTRITO DE BARRANQUITA DE LA PROVINCIA DE LAMAS DEL DEPARTAMENTO DE SAN MARTÍN”</t>
@@ -3411,11 +3411,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="34083187"/>
-        <c:axId val="24043534"/>
+        <c:axId val="13394852"/>
+        <c:axId val="20046577"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="34083187"/>
+        <c:axId val="13394852"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3494,7 +3494,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24043534"/>
+        <c:crossAx val="20046577"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3502,7 +3502,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="24043534"/>
+        <c:axId val="20046577"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="1"/>
@@ -3582,7 +3582,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34083187"/>
+        <c:crossAx val="13394852"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3825,11 +3825,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="24775817"/>
-        <c:axId val="44616564"/>
+        <c:axId val="36555901"/>
+        <c:axId val="82587165"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="24775817"/>
+        <c:axId val="36555901"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3862,7 +3862,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44616564"/>
+        <c:crossAx val="82587165"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3870,7 +3870,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="44616564"/>
+        <c:axId val="82587165"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3913,7 +3913,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="24775817"/>
+        <c:crossAx val="36555901"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4186,11 +4186,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="36404320"/>
-        <c:axId val="25212572"/>
+        <c:axId val="21529918"/>
+        <c:axId val="93846437"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="36404320"/>
+        <c:axId val="21529918"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4223,7 +4223,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25212572"/>
+        <c:crossAx val="93846437"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4231,7 +4231,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="25212572"/>
+        <c:axId val="93846437"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4274,7 +4274,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36404320"/>
+        <c:crossAx val="21529918"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4547,11 +4547,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="50443040"/>
-        <c:axId val="6503093"/>
+        <c:axId val="77022824"/>
+        <c:axId val="29180242"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="50443040"/>
+        <c:axId val="77022824"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4584,7 +4584,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6503093"/>
+        <c:crossAx val="29180242"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4592,7 +4592,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6503093"/>
+        <c:axId val="29180242"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4635,7 +4635,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50443040"/>
+        <c:crossAx val="77022824"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4908,11 +4908,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="19003505"/>
-        <c:axId val="71664288"/>
+        <c:axId val="86855589"/>
+        <c:axId val="66852188"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="19003505"/>
+        <c:axId val="86855589"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4945,7 +4945,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71664288"/>
+        <c:crossAx val="66852188"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4953,7 +4953,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="71664288"/>
+        <c:axId val="66852188"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4996,7 +4996,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19003505"/>
+        <c:crossAx val="86855589"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5658,11 +5658,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="21343222"/>
-        <c:axId val="37489241"/>
+        <c:axId val="11519992"/>
+        <c:axId val="81538335"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="21343222"/>
+        <c:axId val="11519992"/>
         <c:scaling>
           <c:logBase val="10"/>
           <c:orientation val="minMax"/>
@@ -5760,12 +5760,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37489241"/>
+        <c:crossAx val="81538335"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="37489241"/>
+        <c:axId val="81538335"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5853,7 +5853,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21343222"/>
+        <c:crossAx val="11519992"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -7067,11 +7067,11 @@
           </c:yVal>
           <c:smooth val="1"/>
         </c:ser>
-        <c:axId val="20659962"/>
-        <c:axId val="81949912"/>
+        <c:axId val="30993252"/>
+        <c:axId val="10564193"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="20659962"/>
+        <c:axId val="30993252"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:max val="120"/>
@@ -7161,13 +7161,13 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81949912"/>
+        <c:crossAx val="10564193"/>
         <c:crossesAt val="0"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="20"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="81949912"/>
+        <c:axId val="10564193"/>
         <c:scaling>
           <c:orientation val="minMax"/>
           <c:min val="0"/>
@@ -7256,7 +7256,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20659962"/>
+        <c:crossAx val="30993252"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="40"/>
@@ -8087,7 +8087,7 @@
     <mergeCell ref="A16:H16"/>
     <mergeCell ref="A17:H17"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="true"/>
   <pageMargins left="0.7875" right="0.7875" top="0.7875" bottom="0.590277777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">

</xml_diff>